<commit_message>
fix: support unary array expressions
</commit_message>
<xml_diff>
--- a/Freexcel/test-corpus/regressions/formula-cached/excel-cached-formula-array-expressions.xlsx
+++ b/Freexcel/test-corpus/regressions/formula-cached/excel-cached-formula-array-expressions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\anton\Documents\Claude\Freexcel\.worktrees\formula-parity-loop\Freexcel\test-corpus\regressions\formula-cached\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7192E779-5F48-41B0-A1FF-2F0BBBF6EE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{18D368FD-0E52-4848-A8E7-8CD78F014ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43110" yWindow="6315" windowWidth="26610" windowHeight="12075" xr2:uid="{D4ED76E1-2DBE-4809-BB07-01B304B82646}"/>
+    <workbookView xWindow="43110" yWindow="6315" windowWidth="26610" windowHeight="12075" xr2:uid="{1A7D3E0E-5BEE-419D-B86A-5BAC7AD01EA6}"/>
   </bookViews>
   <sheets>
     <sheet name="array-expressions" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>FILTER include array comparison reduced by SUM</t>
   </si>
@@ -49,6 +49,12 @@
   </si>
   <si>
     <t>Less-or-equal array comparison multiplied by values</t>
+  </si>
+  <si>
+    <t>Dynamic array unary minus reduced by SUM</t>
+  </si>
+  <si>
+    <t>Dynamic array percent reduced by SUM</t>
   </si>
 </sst>
 </file>
@@ -399,8 +405,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BDF9702-23B9-4EE8-9202-3DBD8316E6BC}">
-  <dimension ref="A1:E5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5495DF63-FF69-46A7-8E30-E6143BF489B6}">
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.90625" bestFit="1" customWidth="1"/>
@@ -472,6 +478,24 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D6">
+        <f>SUM(-_xlfn.SEQUENCE(2,2))</f>
+        <v>-10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D7">
+        <f>SUM(_xlfn.SEQUENCE(2,2)%)</f>
+        <v>0.1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>